<commit_message>
Improve automation workflow and output handling
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -1,41 +1,83 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Contacts" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    </ext>
+  </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t xml:space="preserve">Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Velmurugan Aircel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hi {name}, this is a test message sent through Playwright.</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="4">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -43,96 +85,61 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="6">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -167,7 +174,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -201,7 +208,7 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -235,205 +242,170 @@
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="50000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="35000">
               <a:schemeClr val="phClr">
                 <a:tint val="37000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:tint val="15000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:shade val="51000"/>
-                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
                 <a:shade val="93000"/>
-                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="94000"/>
-                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="40000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="40000">
               <a:schemeClr val="phClr">
                 <a:tint val="45000"/>
                 <a:shade val="99000"/>
-                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="20000"/>
-                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
-                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="30000"/>
-                <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="50.09"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Message</t>
-        </is>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>9842389755</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>